<commit_message>
Some changes are done not imp
</commit_message>
<xml_diff>
--- a/ResultData/OutputData.xlsx
+++ b/ResultData/OutputData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2483954\IdeaProjects\IdentifyCourses\ResultData\"/>
     </mc:Choice>
@@ -19,7 +19,7 @@
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="96">
   <si>
     <t>Languages Names</t>
   </si>
@@ -290,12 +290,125 @@
   </si>
   <si>
     <t>Beginner · Specialization · 1 - 3 Months</t>
+  </si>
+  <si>
+    <t>English
+(6,179)</t>
+  </si>
+  <si>
+    <t>Kazakh
+(2,727)</t>
+  </si>
+  <si>
+    <t>Spanish
+(2,627)</t>
+  </si>
+  <si>
+    <t>French
+(2,603)</t>
+  </si>
+  <si>
+    <t>German
+(2,548)</t>
+  </si>
+  <si>
+    <t>Arabic
+(2,541)</t>
+  </si>
+  <si>
+    <t>Portuguese
+(1,905)</t>
+  </si>
+  <si>
+    <t>Indonesian
+(1,902)</t>
+  </si>
+  <si>
+    <t>Chinese
+(1,715)</t>
+  </si>
+  <si>
+    <t>Japanese
+(1,675)</t>
+  </si>
+  <si>
+    <t>Korean
+(1,674)</t>
+  </si>
+  <si>
+    <t>Hindi
+(1,640)</t>
+  </si>
+  <si>
+    <t>Thai
+(1,592)</t>
+  </si>
+  <si>
+    <t>Greek
+(1,575)</t>
+  </si>
+  <si>
+    <t>Dutch
+(1,551)</t>
+  </si>
+  <si>
+    <t>Swedish
+(1,537)</t>
+  </si>
+  <si>
+    <t>Vietnamese
+(1,259)</t>
+  </si>
+  <si>
+    <t>Uzbek
+(1,211)</t>
+  </si>
+  <si>
+    <t>Azerbaijani
+(1,086)</t>
+  </si>
+  <si>
+    <t>Urdu
+(935)</t>
+  </si>
+  <si>
+    <t>Bengali
+(932)</t>
+  </si>
+  <si>
+    <t>Oriya
+(190)</t>
+  </si>
+  <si>
+    <t>Persian
+(31)</t>
+  </si>
+  <si>
+    <t>Khmer
+(26)</t>
+  </si>
+  <si>
+    <t>Beginner
+(3,131)</t>
+  </si>
+  <si>
+    <t>Intermediate
+(2,488)</t>
+  </si>
+  <si>
+    <t>Advanced
+(307)</t>
+  </si>
+  <si>
+    <t>Mixed
+(630)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -611,277 +724,277 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>1</v>
+      <c r="A2" t="s" s="0">
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>2</v>
+      <c r="A3" t="s" s="0">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>3</v>
+      <c r="A4" t="s" s="0">
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>4</v>
+      <c r="A5" t="s" s="0">
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>5</v>
+      <c r="A6" t="s" s="0">
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>6</v>
+      <c r="A7" t="s" s="0">
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>7</v>
+      <c r="A8" t="s" s="0">
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>8</v>
+      <c r="A9" t="s" s="0">
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>9</v>
+      <c r="A10" t="s" s="0">
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+      <c r="A11" t="s" s="0">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>11</v>
+      <c r="A12" t="s" s="0">
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>12</v>
+      <c r="A13" t="s" s="0">
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>13</v>
+      <c r="A14" t="s" s="0">
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+      <c r="A15" t="s" s="0">
         <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="A16" t="s" s="0">
         <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>16</v>
+      <c r="A17" t="s" s="0">
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="A18" t="s" s="0">
         <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>18</v>
+      <c r="A19" t="s" s="0">
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="A20" t="s" s="0">
         <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>20</v>
+      <c r="A21" t="s" s="0">
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>21</v>
+      <c r="A22" t="s" s="0">
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="A23" t="s" s="0">
         <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>23</v>
+      <c r="A24" t="s" s="0">
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+      <c r="A25" t="s" s="0">
         <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>25</v>
+      <c r="A26" t="s" s="0">
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>26</v>
+      <c r="A27" t="s" s="0">
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>27</v>
+      <c r="A28" t="s" s="0">
+        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>28</v>
+      <c r="A29" t="s" s="0">
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>29</v>
+      <c r="A30" t="s" s="0">
+        <v>89</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+      <c r="A31" t="s" s="0">
         <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+      <c r="A32" t="s" s="0">
         <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>32</v>
+      <c r="A33" t="s" s="0">
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>33</v>
+      <c r="A34" t="s" s="0">
+        <v>91</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+      <c r="A35" t="s" s="0">
         <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+      <c r="A36" t="s" s="0">
         <v>35</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+      <c r="A37" t="s" s="0">
         <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+      <c r="A38" t="s" s="0">
         <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+      <c r="A39" t="s" s="0">
         <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+      <c r="A40" t="s" s="0">
         <v>39</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+      <c r="A41" t="s" s="0">
         <v>40</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+      <c r="A42" t="s" s="0">
         <v>41</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+      <c r="A43" t="s" s="0">
         <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+      <c r="A44" t="s" s="0">
         <v>43</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+      <c r="A45" t="s" s="0">
         <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+      <c r="A46" t="s" s="0">
         <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+      <c r="A47" t="s" s="0">
         <v>46</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+      <c r="A48" t="s" s="0">
         <v>47</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+      <c r="A49" t="s" s="0">
         <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+      <c r="A50" t="s" s="0">
         <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
+      <c r="A51" t="s" s="0">
         <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
+      <c r="A52" t="s" s="0">
         <v>51</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
+      <c r="A53" t="s" s="0">
         <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
+      <c r="A54" t="s" s="0">
         <v>53</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
+      <c r="A55" t="s" s="0">
         <v>54</v>
       </c>
     </row>
@@ -896,28 +1009,28 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>56</v>
+      <c r="A2" t="s" s="0">
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>57</v>
+      <c r="A3" t="s" s="0">
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>58</v>
+      <c r="A4" t="s" s="0">
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>59</v>
+      <c r="A5" t="s" s="0">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -930,41 +1043,41 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="56" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="56.0"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="24.6328125"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="33.36328125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>60</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>61</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>63</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>65</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" t="s" s="0">
         <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>64</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>65</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" t="s" s="0">
         <v>67</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel file path made dynamic
</commit_message>
<xml_diff>
--- a/ResultData/OutputData.xlsx
+++ b/ResultData/OutputData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="133">
   <si>
     <t>Languages Names</t>
   </si>
@@ -402,6 +402,150 @@
   <si>
     <t>Mixed
 (630)</t>
+  </si>
+  <si>
+    <t>English
+(6,189)</t>
+  </si>
+  <si>
+    <t>Kazakh
+(2,725)</t>
+  </si>
+  <si>
+    <t>Spanish
+(2,631)</t>
+  </si>
+  <si>
+    <t>French
+(2,608)</t>
+  </si>
+  <si>
+    <t>German
+(2,550)</t>
+  </si>
+  <si>
+    <t>Arabic
+(2,543)</t>
+  </si>
+  <si>
+    <t>Chinese
+(1,717)</t>
+  </si>
+  <si>
+    <t>Russian
+(1,693)</t>
+  </si>
+  <si>
+    <t>Korean
+(1,673)</t>
+  </si>
+  <si>
+    <t>Japanese
+(1,671)</t>
+  </si>
+  <si>
+    <t>Hindi
+(1,637)</t>
+  </si>
+  <si>
+    <t>Italian
+(1,611)</t>
+  </si>
+  <si>
+    <t>Turkish
+(1,608)</t>
+  </si>
+  <si>
+    <t>Thai
+(1,589)</t>
+  </si>
+  <si>
+    <t>Ukrainian
+(1,589)</t>
+  </si>
+  <si>
+    <t>Greek
+(1,572)</t>
+  </si>
+  <si>
+    <t>Polish
+(1,551)</t>
+  </si>
+  <si>
+    <t>Dutch
+(1,548)</t>
+  </si>
+  <si>
+    <t>Swedish
+(1,534)</t>
+  </si>
+  <si>
+    <t>Hungarian
+(1,453)</t>
+  </si>
+  <si>
+    <t>Vietnamese
+(1,255)</t>
+  </si>
+  <si>
+    <t>Pushto
+(1,247)</t>
+  </si>
+  <si>
+    <t>Uzbek
+(1,210)</t>
+  </si>
+  <si>
+    <t>Azerbaijani
+(1,083)</t>
+  </si>
+  <si>
+    <t>Urdu
+(932)</t>
+  </si>
+  <si>
+    <t>Bengali
+(929)</t>
+  </si>
+  <si>
+    <t>Oriya
+(188)</t>
+  </si>
+  <si>
+    <t>Haitian (Haitian Creole)
+(81)</t>
+  </si>
+  <si>
+    <t>Beginner
+(3,137)</t>
+  </si>
+  <si>
+    <t>Intermediate
+(2,492)</t>
+  </si>
+  <si>
+    <t>Mixed
+(631)</t>
+  </si>
+  <si>
+    <t>How to Get Into Web Development</t>
+  </si>
+  <si>
+    <t>Introduction to Web Development</t>
+  </si>
+  <si>
+    <t>4.1
+Rating, 4.1 out of 5 stars</t>
+  </si>
+  <si>
+    <t>4.6
+Rating, 4.6 out of 5 stars</t>
+  </si>
+  <si>
+    <t>Beginner · Course · 1 - 4 Weeks</t>
+  </si>
+  <si>
+    <t>Beginner · Course · 1 - 3 Months</t>
   </si>
 </sst>
 </file>
@@ -730,37 +874,37 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>68</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>69</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s" s="0">
-        <v>70</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s" s="0">
-        <v>71</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s" s="0">
-        <v>72</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s" s="0">
-        <v>73</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s" s="0">
-        <v>74</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
@@ -770,107 +914,107 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s" s="0">
-        <v>76</v>
+        <v>102</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s" s="0">
-        <v>10</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s" s="0">
-        <v>77</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s" s="0">
-        <v>78</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s" s="0">
-        <v>79</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s" s="0">
-        <v>14</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s" s="0">
-        <v>15</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s" s="0">
-        <v>80</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s" s="0">
-        <v>17</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s" s="0">
-        <v>81</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s" s="0">
-        <v>19</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s" s="0">
-        <v>82</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s" s="0">
-        <v>83</v>
+        <v>114</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s" s="0">
-        <v>22</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s" s="0">
-        <v>84</v>
+        <v>116</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s" s="0">
-        <v>24</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s" s="0">
-        <v>85</v>
+        <v>118</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s" s="0">
-        <v>86</v>
+        <v>119</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s" s="0">
-        <v>87</v>
+        <v>120</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s" s="0">
-        <v>88</v>
+        <v>121</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s" s="0">
-        <v>89</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
@@ -880,7 +1024,7 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s" s="0">
-        <v>31</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
@@ -890,7 +1034,7 @@
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s" s="0">
-        <v>91</v>
+        <v>33</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
@@ -1015,12 +1159,12 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>92</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>93</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
@@ -1030,7 +1174,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s" s="0">
-        <v>95</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1061,24 +1205,24 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>63</v>
+        <v>127</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>65</v>
+        <v>129</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>66</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>64</v>
+        <v>128</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>65</v>
+        <v>130</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>67</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
All test cases added in one test case no 8
</commit_message>
<xml_diff>
--- a/ResultData/OutputData.xlsx
+++ b/ResultData/OutputData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="151">
   <si>
     <t>Languages Names</t>
   </si>
@@ -546,6 +546,76 @@
   </si>
   <si>
     <t>Beginner · Course · 1 - 3 Months</t>
+  </si>
+  <si>
+    <t>English
+(6,199)</t>
+  </si>
+  <si>
+    <t>Kazakh
+(2,729)</t>
+  </si>
+  <si>
+    <t>Spanish
+(2,632)</t>
+  </si>
+  <si>
+    <t>French
+(2,611)</t>
+  </si>
+  <si>
+    <t>German
+(2,554)</t>
+  </si>
+  <si>
+    <t>Portuguese
+(1,909)</t>
+  </si>
+  <si>
+    <t>Indonesian
+(1,904)</t>
+  </si>
+  <si>
+    <t>Japanese
+(1,677)</t>
+  </si>
+  <si>
+    <t>Italian
+(1,615)</t>
+  </si>
+  <si>
+    <t>Turkish
+(1,611)</t>
+  </si>
+  <si>
+    <t>Ukrainian
+(1,592)</t>
+  </si>
+  <si>
+    <t>Pushto
+(1,249)</t>
+  </si>
+  <si>
+    <t>Uzbek
+(1,212)</t>
+  </si>
+  <si>
+    <t>Beginner
+(3,147)</t>
+  </si>
+  <si>
+    <t>Mixed
+(628)</t>
+  </si>
+  <si>
+    <t>Full-Stack Web Development: PHP, HTML, CSS &amp; JavaScript</t>
+  </si>
+  <si>
+    <t>Full-Stack Web Development</t>
+  </si>
+  <si>
+    <t>4
+Rating, 4 out of 5 stars</t>
   </si>
 </sst>
 </file>
@@ -874,42 +944,42 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>96</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>97</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s" s="0">
-        <v>98</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s" s="0">
-        <v>99</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s" s="0">
-        <v>100</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s" s="0">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s" s="0">
-        <v>7</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s" s="0">
-        <v>75</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
@@ -919,102 +989,102 @@
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s" s="0">
-        <v>103</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s" s="0">
-        <v>104</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s" s="0">
-        <v>105</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s" s="0">
-        <v>106</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s" s="0">
-        <v>107</v>
+        <v>141</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s" s="0">
-        <v>108</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s" s="0">
-        <v>109</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s" s="0">
-        <v>110</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s" s="0">
-        <v>111</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s" s="0">
-        <v>112</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s" s="0">
-        <v>113</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s" s="0">
-        <v>114</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s" s="0">
-        <v>115</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s" s="0">
-        <v>116</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s" s="0">
-        <v>117</v>
+        <v>144</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s" s="0">
-        <v>118</v>
+        <v>145</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s" s="0">
-        <v>119</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s" s="0">
-        <v>120</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s" s="0">
-        <v>121</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s" s="0">
-        <v>122</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
@@ -1024,7 +1094,7 @@
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s" s="0">
-        <v>123</v>
+        <v>31</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
@@ -1159,22 +1229,22 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>124</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>125</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s" s="0">
-        <v>94</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s" s="0">
-        <v>126</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -1205,24 +1275,24 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>131</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>130</v>
+        <v>65</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>132</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
some changes are done like actions->javascriptexcutor
</commit_message>
<xml_diff>
--- a/ResultData/OutputData.xlsx
+++ b/ResultData/OutputData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="172">
   <si>
     <t>Languages Names</t>
   </si>
@@ -616,6 +616,88 @@
   <si>
     <t>4
 Rating, 4 out of 5 stars</t>
+  </si>
+  <si>
+    <t>Language List</t>
+  </si>
+  <si>
+    <t>Level List</t>
+  </si>
+  <si>
+    <t>Beginner
+(2,901)</t>
+  </si>
+  <si>
+    <t>Intermediate
+(2,387)</t>
+  </si>
+  <si>
+    <t>Advanced
+(301)</t>
+  </si>
+  <si>
+    <t>Mixed
+(610)</t>
+  </si>
+  <si>
+    <t>English
+(6,216)</t>
+  </si>
+  <si>
+    <t>Kazakh
+(2,730)</t>
+  </si>
+  <si>
+    <t>Spanish
+(2,637)</t>
+  </si>
+  <si>
+    <t>Arabic
+(2,547)</t>
+  </si>
+  <si>
+    <t>Portuguese
+(1,911)</t>
+  </si>
+  <si>
+    <t>Indonesian
+(1,905)</t>
+  </si>
+  <si>
+    <t>Chinese
+(1,719)</t>
+  </si>
+  <si>
+    <t>Russian
+(1,697)</t>
+  </si>
+  <si>
+    <t>Polish
+(1,553)</t>
+  </si>
+  <si>
+    <t>Hungarian
+(1,459)</t>
+  </si>
+  <si>
+    <t>Urdu
+(934)</t>
+  </si>
+  <si>
+    <t>Bengali
+(931)</t>
+  </si>
+  <si>
+    <t>Beginner
+(3,153)</t>
+  </si>
+  <si>
+    <t>Intermediate
+(2,504)</t>
+  </si>
+  <si>
+    <t>Advanced
+(310)</t>
   </si>
 </sst>
 </file>
@@ -944,17 +1026,17 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>133</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>134</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s" s="0">
-        <v>135</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
@@ -969,27 +1051,27 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s" s="0">
-        <v>6</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s" s="0">
-        <v>138</v>
+        <v>161</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s" s="0">
-        <v>139</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s" s="0">
-        <v>102</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s" s="0">
-        <v>10</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
@@ -1009,12 +1091,12 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s" s="0">
-        <v>141</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s" s="0">
-        <v>142</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
@@ -1024,7 +1106,7 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s" s="0">
-        <v>143</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
@@ -1034,22 +1116,22 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s" s="0">
-        <v>19</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s" s="0">
-        <v>82</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s" s="0">
-        <v>83</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s" s="0">
-        <v>22</v>
+        <v>166</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
@@ -1059,7 +1141,7 @@
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s" s="0">
-        <v>144</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
@@ -1069,17 +1151,17 @@
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s" s="0">
-        <v>26</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s" s="0">
-        <v>27</v>
+        <v>167</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s" s="0">
-        <v>28</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
@@ -1229,22 +1311,22 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>146</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>93</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s" s="0">
-        <v>58</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s" s="0">
-        <v>147</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1275,21 +1357,21 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>148</v>
+        <v>63</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>150</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>65</v>
+        <v>150</v>
       </c>
       <c r="C3" t="s" s="0">
         <v>67</v>

</xml_diff>

<commit_message>
Some changes are added
</commit_message>
<xml_diff>
--- a/ResultData/OutputData.xlsx
+++ b/ResultData/OutputData.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="205">
   <si>
     <t>Languages Names</t>
   </si>
@@ -698,6 +698,138 @@
   <si>
     <t>Advanced
 (310)</t>
+  </si>
+  <si>
+    <t>English
+(6,245)</t>
+  </si>
+  <si>
+    <t>Kazakh
+(2,740)</t>
+  </si>
+  <si>
+    <t>Spanish
+(2,645)</t>
+  </si>
+  <si>
+    <t>French
+(2,618)</t>
+  </si>
+  <si>
+    <t>German
+(2,561)</t>
+  </si>
+  <si>
+    <t>Arabic
+(2,554)</t>
+  </si>
+  <si>
+    <t>Portuguese
+(1,919)</t>
+  </si>
+  <si>
+    <t>Indonesian
+(1,912)</t>
+  </si>
+  <si>
+    <t>Chinese
+(1,727)</t>
+  </si>
+  <si>
+    <t>Russian
+(1,705)</t>
+  </si>
+  <si>
+    <t>Korean
+(1,686)</t>
+  </si>
+  <si>
+    <t>Japanese
+(1,683)</t>
+  </si>
+  <si>
+    <t>Hindi
+(1,652)</t>
+  </si>
+  <si>
+    <t>Italian
+(1,623)</t>
+  </si>
+  <si>
+    <t>Turkish
+(1,619)</t>
+  </si>
+  <si>
+    <t>Thai
+(1,601)</t>
+  </si>
+  <si>
+    <t>Ukrainian
+(1,600)</t>
+  </si>
+  <si>
+    <t>Greek
+(1,584)</t>
+  </si>
+  <si>
+    <t>Polish
+(1,562)</t>
+  </si>
+  <si>
+    <t>Dutch
+(1,559)</t>
+  </si>
+  <si>
+    <t>Swedish
+(1,545)</t>
+  </si>
+  <si>
+    <t>Hungarian
+(1,461)</t>
+  </si>
+  <si>
+    <t>Vietnamese
+(1,267)</t>
+  </si>
+  <si>
+    <t>Pushto
+(1,258)</t>
+  </si>
+  <si>
+    <t>Uzbek
+(1,223)</t>
+  </si>
+  <si>
+    <t>Azerbaijani
+(1,095)</t>
+  </si>
+  <si>
+    <t>Urdu
+(938)</t>
+  </si>
+  <si>
+    <t>Bengali
+(935)</t>
+  </si>
+  <si>
+    <t>Malay
+(146)</t>
+  </si>
+  <si>
+    <t>Swahili
+(1)</t>
+  </si>
+  <si>
+    <t>Beginner
+(3,176)</t>
+  </si>
+  <si>
+    <t>Intermediate
+(2,507)</t>
+  </si>
+  <si>
+    <t>Mixed
+(633)</t>
   </si>
 </sst>
 </file>
@@ -1026,142 +1158,142 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>157</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>158</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s" s="0">
-        <v>159</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s" s="0">
-        <v>136</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s" s="0">
-        <v>137</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s" s="0">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s" s="0">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s" s="0">
-        <v>162</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s" s="0">
-        <v>163</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s" s="0">
-        <v>164</v>
+        <v>181</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s" s="0">
-        <v>140</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s" s="0">
-        <v>12</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s" s="0">
-        <v>79</v>
+        <v>184</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s" s="0">
-        <v>14</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s" s="0">
-        <v>15</v>
+        <v>186</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s" s="0">
-        <v>80</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s" s="0">
-        <v>17</v>
+        <v>188</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s" s="0">
-        <v>81</v>
+        <v>189</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s" s="0">
-        <v>165</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s" s="0">
-        <v>20</v>
+        <v>191</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s" s="0">
-        <v>21</v>
+        <v>192</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s" s="0">
-        <v>166</v>
+        <v>193</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s" s="0">
-        <v>84</v>
+        <v>194</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s" s="0">
-        <v>24</v>
+        <v>195</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s" s="0">
-        <v>145</v>
+        <v>196</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s" s="0">
-        <v>86</v>
+        <v>197</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s" s="0">
-        <v>167</v>
+        <v>198</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s" s="0">
-        <v>168</v>
+        <v>199</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
@@ -1171,7 +1303,7 @@
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s" s="0">
-        <v>30</v>
+        <v>200</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
@@ -1261,32 +1393,32 @@
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s" s="0">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s" s="0">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="s" s="0">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="s" s="0">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s" s="0">
-        <v>53</v>
+        <v>201</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
@@ -1311,12 +1443,12 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>169</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>170</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
@@ -1326,7 +1458,7 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s" s="0">
-        <v>126</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -1357,24 +1489,24 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
-        <v>63</v>
+        <v>149</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>65</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s" s="0">
-        <v>148</v>
+        <v>63</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>150</v>
+        <v>65</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>